<commit_message>
data(uae): document review + first two listings — registration proof status (management-confirmed, proof not in files), SKINLAB scope (CEEL Pure Rosemary Water only), trademark = application by natural person + unsigned authorization draft, EANs from packaging artwork, account-vs-product split in 4-platform checklists — no import
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/b2b/uae/commercial_kit_2026-10-09/LOWES_UAE_Readiness_and_Products_2026-10-09.xlsx
+++ b/data/b2b/uae/commercial_kit_2026-10-09/LOWES_UAE_Readiness_and_Products_2026-10-09.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet name="جاهزية" sheetId="1" r:id="rId1"/>
     <sheet name="المنتجات 26" sheetId="2" r:id="rId2"/>
+    <sheet name="أول منتجين" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -398,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -611,7 +612,7 @@
         <v>management_confirmed_proof_not_in_files</v>
       </c>
       <c r="C8" t="str">
-        <v>**أكدت الإدارة أن التسجيل مكتمل؛ إثبات التسجيل (شهادات/أرقام) لم يُعثر عليه في ملفات المشروع.** الموجود محلياً: فهرس شهادات يشير لملف اختبارات الـ26 منتجاً (استقرار، تحدي/حفظ، ميكروبيولوجي — 80+ وثيقة) على Google Drive، وصور تسجيل ÜTS التركي</v>
+        <v>**الإدارة تؤكد اكتمال التسجيل، لكن إثبات التسجيل لم يُعثر عليه في الملفات المتاحة.** بحث 9/10/2026 (Montaji/بلدية دبي/ECAS/ESMA/MoIAT/أرقام): لا نتيجة. الموجود: صور ÜTS تركية لـ7 منتجات (ليست إماراتية)، وفهرس يشير لملف اختبارات الـ26 منتجاً على Drive</v>
       </c>
       <c r="D8" t="str">
         <v>إفادة الإدارة (9/10/2026) + غرفة بيانات المستثمرين/03_الشهادات/00_فهرس الشهادات.pdf</v>
@@ -626,7 +627,7 @@
         <v>قائمة SKUs المسجلة وأرقامها والجهة (مثلاً Montaji/بلدية دبي)</v>
       </c>
       <c r="H8" t="str">
-        <v>تزويد نسخة الشهادات أو أرقام التسجيل لكل SKU — **لا إعادة تسجيل**</v>
+        <v>نسخة الشهادات أو أرقامها لكل SKU — لا إعادة تسجيل</v>
       </c>
       <c r="I8" t="str">
         <v>الإدارة</v>
@@ -637,13 +638,13 @@
         <v>باركودات GTIN/EAN-13</v>
       </c>
       <c r="B9" t="str">
-        <v>not_found_in_project_files</v>
+        <v>available_in_project_files (partial: 3 SKUs)</v>
       </c>
       <c r="C9" t="str">
-        <v>حقل «barcode» بقاعدة Brand Kit يحمل رموزاً داخلية (LW-…) ورموز الكتالوج (LSK-…)؛ لا أرقام EAN بالكتالوجات الثلاثة ولا بملفات المشروع — قد تكون على العبوات الفعلية</v>
+        <v>EAN-13 مطبوع على تصاميم العبوات بالملفات (رقم التحقق صحيح): Vitamin C Serum 8684272100419 · Rosemary Hair Oil 8684272100471 · Pore Tightening Toner 8684149133717. باقي الـ23: غير موجود بالملفات (التصاميم غير قابلة للقراءة آلياً)</v>
       </c>
       <c r="D9" t="str">
-        <v>LOWES Brand Kit/system/src/db/database.js + كتالوجات غرفة البيانات (بحث عن 13 رقماً: لا نتيجة)</v>
+        <v>04 - السوشال ميديا والمحتوى/صور المنتجات ومعلومات عنها/… Box.pdf / تفاصيل المنتج.pdf</v>
       </c>
       <c r="E9" t="str">
         <v>listing</v>
@@ -652,10 +653,10 @@
         <v>Amazon.ae (GTIN أو إعفاء)؛ noon (باركود على كل وحدة للـFBN/FBP؛ باركود مخصص مسموح للإدراج بحسب صفحة رسمية مفهرسة)؛ Begad/Dayjour (غير منصوص)</v>
       </c>
       <c r="G9" t="str">
-        <v>هل للمنتجات EAN مطبوع على العبوة؟ ومن مالكه (CEELLO أم العلامة)؟</v>
+        <v>الطباعة على العبوة الحالية + صاحب ترخيص بادئة GS1 (8684272 و8684149 مختلفتان)</v>
       </c>
       <c r="H9" t="str">
-        <v>فحص عبوة من كل SKU وتسجيل الباركود المطبوع إن وُجد؛ وإلا قرار: GS1 UAE أم إعفاء Amazon</v>
+        <v>تأكيد من العبوات الفعلية وجهة إصدار الباركود؛ استكمال الـ23 من العبوات</v>
       </c>
       <c r="I9" t="str">
         <v>الإدارة</v>
@@ -669,7 +670,7 @@
         <v>available_in_project_files (partial)</v>
       </c>
       <c r="C10" t="str">
-        <v>وثيقة طلب العلامة التركية «lowe's profesyonel» (طلب 2024/085278، صنف 03 و35) — **مالك الطلب بالوثيقة شخص طبيعي وليس الكيان التركي**. لا خطاب تفويض للكيان الإماراتي بملفات المشروع</v>
+        <v>الملف الموجود **طلب تسجيل** (MARKA BAŞVURUSU 2024/085278، 04.07.2024، صنف 03 و35) — مالك الطلب **شخص طبيعي** (البيانات بالوثيقة، لم تُنقل). لا شهادة تسجيل نهائية لـLOWE'S ولا تسجيل إماراتي بالملفات. مسودة خطاب تفويض جاهزة غير موقّعة</v>
       </c>
       <c r="D10" t="str">
         <v>غرفة بيانات المستثمرين/02_العلامات التجارية/شهادة تسجيل علامة LOWES - تركيا.pdf</v>
@@ -684,7 +685,7 @@
         <v>حالة التسجيل النهائي، ومن يوقّع التفويض (مالك العلامة الوارد بالوثيقة)</v>
       </c>
       <c r="H10" t="str">
-        <v>تحضير خطاب تفويض من مالك العلامة إلى Lowes Professional L.L.C-FZ (قرار إداري)</v>
+        <v>تأكيد المالك الحالي/حالة التسجيل؛ مراجعة وتوقيع المسودة من صاحب الصلاحية</v>
       </c>
       <c r="I10" t="str">
         <v>الإدارة</v>
@@ -698,7 +699,7 @@
         <v>available_in_project_files</v>
       </c>
       <c r="C11" t="str">
-        <v>بيان شراكة تصنيعية: CEELLO KOZMETİK (أفيون قره حصار) مصنّع تعاقدي، تركيبات LOWE'S مطابقة 100% لتركيبات CEEL/CEELLO</v>
+        <v>«بيان الشراكة التصنيعية» **وثيقة أعدّتها الشركة** (مادة معرض دمشق 2026) تقول إن CEELLO مصنّع تعاقدي والتركيبات مطابقة 100%، وتوصي بالحصول على كتاب رسمي من CEELLO — **لا إقرار صادر عن CEELLO بالملفات**</v>
       </c>
       <c r="D11" t="str">
         <v>غرفة بيانات المستثمرين/03_الشهادات/01_بيان الشراكة التصنيعية وتوثيق الشهادات.pdf</v>
@@ -727,7 +728,7 @@
         <v>available_in_project_files</v>
       </c>
       <c r="C12" t="str">
-        <v>تقرير SKINLAB P.S.A. (كراكوف) 20/03/2026: «The CEEL Pure Rosemary Water» — زيادة كثافة الشعر 15.53% بعد 8 أسابيع، 30 متطوعة، بلا آثار جانبية، معتمد من د. Barbara Wnuk. **المنتج المختبَر يحمل اسم CEEL (علامة المصنّع)** — يُستخدم لـLOWE'S Pure Rosemary Water استناداً لبيان تطابق التركيبات</v>
+        <v>SKINLAB P.S.A. 20/03/2026: المنتج المختبَر «The CEEL Pure Rosemary Water» (طلب CEELLO) — +15.53% كثافة شعر، 30 متطوعة، 8 أسابيع. **يقابل LOWE'S Pure Rosemary Water (LHR-TNR-01) فقط، ولا يُنسب له رسمياً قبل إقرار CEELLO؛ لا ينطبق على Rosemary Hair Oil**</v>
       </c>
       <c r="D12" t="str">
         <v>غرفة بيانات المستثمرين/03_الشهادات/تقرير الفحص والشهادة (AplAppRep).pdf</v>
@@ -742,7 +743,7 @@
         <v>قبول المنصات لادعاء مبني على اختبار باسم المصنّع</v>
       </c>
       <c r="H12" t="str">
-        <v>إرفاق التقرير + بيان التطابق معاً عند استخدام الادعاء</v>
+        <v>طلب إقرار CEELLO المكتوب بالتطابق قبل استخدام النتائج</v>
       </c>
       <c r="I12" t="str">
         <v>فريق التسجيل</v>
@@ -893,9 +894,96 @@
         <v>الإدارة</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>جهة الملصق على العبوات</v>
+      </c>
+      <c r="B18" t="str">
+        <v>available_in_project_files</v>
+      </c>
+      <c r="C18" t="str">
+        <v>علبتا Vitamin C وRosemary Hair Oil تذكران «L B İÇ VE DIŞ TİCARET KOZMETİK A.Ş., Kadıköy/İstanbul» — يختلف عن الكيانين المسجلين بـABOS</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Box.pdf للمنتجين</v>
+      </c>
+      <c r="E18" t="str">
+        <v>listing + التطابق التنظيمي</v>
+      </c>
+      <c r="F18" t="str">
+        <v>كل المنصات/الجهات التنظيمية</v>
+      </c>
+      <c r="G18" t="str">
+        <v>صفة هذه الجهة (مستورد/مسؤول/مالك علامة)</v>
+      </c>
+      <c r="H18" t="str">
+        <v>توضيح الإدارة</v>
+      </c>
+      <c r="I18" t="str">
+        <v>الإدارة</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>تقارير الاختبار لكل SKU</v>
+      </c>
+      <c r="B19" t="str">
+        <v>available_in_project_files (partial: 10 SKUs)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Stability + Challenge + Microbiological باسم LOWE'S لـ10 منتجات محلياً؛ غير موجودة محلياً لـVitamin C وRosemary Hair Oil (الفهرس يشير إلى Drive)</v>
+      </c>
+      <c r="D19" t="str">
+        <v>04 - السوشال ميديا والمحتوى/صور المنتجات ومعلومات عنها/</v>
+      </c>
+      <c r="E19" t="str">
+        <v>ملف المورد والتسجيل</v>
+      </c>
+      <c r="F19" t="str">
+        <v>الصيدليات والمتاجر</v>
+      </c>
+      <c r="G19" t="str">
+        <v>—</v>
+      </c>
+      <c r="H19" t="str">
+        <v>تنزيل ملفات Drive للمنتجين الأولين إن طُلبت</v>
+      </c>
+      <c r="I19" t="str">
+        <v>فريق التسجيل</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>اتساق بيانات المنتج (INCI والادعاءات)</v>
+      </c>
+      <c r="B20" t="str">
+        <v>available_in_project_files (conflicts)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Rosemary Hair Oil: INCI العلبة ≠ ملف التفاصيل؛ «Biotin» على الواجهة غير موجود بـINCI. Vitamin C: 2% منسوبة لـFerulic بالعلبة ولـB5 بملف التفاصيل</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Box.pdf + تفاصيل المنتج.pdf</v>
+      </c>
+      <c r="E20" t="str">
+        <v>listing</v>
+      </c>
+      <c r="F20" t="str">
+        <v>كل المنصات</v>
+      </c>
+      <c r="G20" t="str">
+        <v>تأكيد المصنّع</v>
+      </c>
+      <c r="H20" t="str">
+        <v>حسم مع CEELLO قبل الإدراج؛ استخدام نص العلبة مؤقتاً لفيتامين سي</v>
+      </c>
+      <c r="I20" t="str">
+        <v>الإدارة</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I20"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -971,7 +1059,7 @@
         <v>LOWES Brand Kit/assets/products_web/fcg01.png</v>
       </c>
       <c r="I2" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J2" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1012,7 +1100,7 @@
         <v>LOWES Brand Kit/assets/products_web/fcg02.png</v>
       </c>
       <c r="I3" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J3" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1053,7 +1141,7 @@
         <v>LOWES Brand Kit/assets/products_web/tnr01.png</v>
       </c>
       <c r="I4" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>8684149133717 (Pore Tightening Toner تفاصيل المنتج.pdf) — من تصميم العبوة؛ ترخيص GS1 والطباعة الحالية يُتحقق منهما</v>
       </c>
       <c r="J4" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1094,7 +1182,7 @@
         <v>LOWES Brand Kit/assets/products_web/pel01.png</v>
       </c>
       <c r="I5" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J5" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1135,7 +1223,7 @@
         <v>LOWES Brand Kit/assets/products_web/ser01.png</v>
       </c>
       <c r="I6" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>8684272100419 (Vitamin C Serum - Box.pdf) — من تصميم العبوة؛ ترخيص GS1 والطباعة الحالية يُتحقق منهما</v>
       </c>
       <c r="J6" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1176,7 +1264,7 @@
         <v>LOWES Brand Kit/assets/products_web/ser02.png</v>
       </c>
       <c r="I7" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J7" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1217,7 +1305,7 @@
         <v>LOWES Brand Kit/assets/products_web/ser03.png</v>
       </c>
       <c r="I8" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J8" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1258,7 +1346,7 @@
         <v>LOWES Brand Kit/assets/products_web/ser04.png</v>
       </c>
       <c r="I9" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J9" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1299,7 +1387,7 @@
         <v>LOWES Brand Kit/assets/products_web/ser05.png</v>
       </c>
       <c r="I10" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J10" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1340,7 +1428,7 @@
         <v>LOWES Brand Kit/assets/products_web/ser06.png</v>
       </c>
       <c r="I11" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J11" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1381,7 +1469,7 @@
         <v>LOWES Brand Kit/assets/products_web/ser07.png</v>
       </c>
       <c r="I12" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J12" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1422,7 +1510,7 @@
         <v>LOWES Brand Kit/assets/products_web/crm01.png</v>
       </c>
       <c r="I13" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J13" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1463,7 +1551,7 @@
         <v>LOWES Brand Kit/assets/products_web/crm04.png</v>
       </c>
       <c r="I14" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J14" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1504,7 +1592,7 @@
         <v>LOWES Brand Kit/assets/products_web/crm02.png</v>
       </c>
       <c r="I15" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J15" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1545,7 +1633,7 @@
         <v>LOWES Brand Kit/assets/products_web/sun01.png</v>
       </c>
       <c r="I16" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J16" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1586,7 +1674,7 @@
         <v>LOWES Brand Kit/assets/products_web/sun02.png</v>
       </c>
       <c r="I17" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J17" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1627,7 +1715,7 @@
         <v>LOWES Brand Kit/assets/products_web/msk01.png</v>
       </c>
       <c r="I18" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J18" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1668,7 +1756,7 @@
         <v>LOWES Brand Kit/assets/products_web/tnr02.png</v>
       </c>
       <c r="I19" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J19" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1709,7 +1797,7 @@
         <v>LOWES Brand Kit/assets/products_web/ser08.png</v>
       </c>
       <c r="I20" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J20" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1750,7 +1838,7 @@
         <v>LOWES Brand Kit/assets/products_web/crm03.png</v>
       </c>
       <c r="I21" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J21" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1791,7 +1879,7 @@
         <v>LOWES Brand Kit/assets/products_web/shm01.png</v>
       </c>
       <c r="I22" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J22" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1832,7 +1920,7 @@
         <v>LOWES Brand Kit/assets/products_web/lhrtnr01.png</v>
       </c>
       <c r="I23" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J23" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1873,7 +1961,7 @@
         <v>LOWES Brand Kit/assets/products_web/oil01.png</v>
       </c>
       <c r="I24" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>8684272100471 (Rosemary Hair Oil - Box (1).pdf) — من تصميم العبوة؛ ترخيص GS1 والطباعة الحالية يُتحقق منهما</v>
       </c>
       <c r="J24" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1914,7 +2002,7 @@
         <v>LOWES Brand Kit/assets/products_web/brd01.png</v>
       </c>
       <c r="I25" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J25" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1955,7 +2043,7 @@
         <v>LOWES Brand Kit/assets/products_web/bodygel.png</v>
       </c>
       <c r="I26" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J26" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -1996,7 +2084,7 @@
         <v>LOWES Brand Kit/assets/products_web/foot01.png</v>
       </c>
       <c r="I27" t="str">
-        <v>غير موجود في ملفات المشروع (حقل barcode بقاعدة Brand Kit = رمز داخلي LW-…؛ قد يكون EAN مطبوعاً على العبوة — يُتحقق)</v>
+        <v>غير موجود في ملفات المشروع (التصميم غير قابل للقراءة آلياً أو غير موجود) — يُتحقق من العبوة</v>
       </c>
       <c r="J27" t="str">
         <v>Made in Türkiye · EU 1223/2009 (مذكوران بالكتالوج)</v>
@@ -2016,4 +2104,93 @@
     <ignoredError numberStoredAsText="1" sqref="A1:M27"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>product</v>
+      </c>
+      <c r="B1" t="str">
+        <v>catalog_code</v>
+      </c>
+      <c r="C1" t="str">
+        <v>sku</v>
+      </c>
+      <c r="D1" t="str">
+        <v>ean</v>
+      </c>
+      <c r="E1" t="str">
+        <v>size</v>
+      </c>
+      <c r="F1" t="str">
+        <v>inci</v>
+      </c>
+      <c r="G1" t="str">
+        <v>uae_registration</v>
+      </c>
+      <c r="H1" t="str">
+        <v>before_publishing</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Vitamin C Serum</v>
+      </c>
+      <c r="B2" t="str">
+        <v>LSK-SER-01</v>
+      </c>
+      <c r="C2" t="str">
+        <v>LW-SR-101</v>
+      </c>
+      <c r="D2" t="str">
+        <v>8684272100419</v>
+      </c>
+      <c r="E2" t="str">
+        <v>30 ml (1.00 fl.oz)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Aqua, Ascorbic Acid, Panthenol, Ferulic Acid, Glycerin, Glutathione, Phenoxyethanol, Ethylhexylglycerin.</v>
+      </c>
+      <c r="G2" t="str">
+        <v>الإدارة تؤكد اكتمال التسجيل، لكن إثبات التسجيل لم يُعثر عليه في الملفات المتاحة</v>
+      </c>
+      <c r="H2" t="str">
+        <v>UAE price (AED) approved · registration proof copy linked to this SKU · confirm EAN on current box + GS1 licensee · confirm label company (L B İç ve Dış Ticaret Kozmetik A.Ş.) role · Amazon: category approval for topicals · brand authorization letter if the platform asks (noon gated brands / Amazon brand approval)</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Rosemary Hair Oil</v>
+      </c>
+      <c r="B3" t="str">
+        <v>LHR-OIL-01</v>
+      </c>
+      <c r="C3" t="str">
+        <v>LW-HR-803</v>
+      </c>
+      <c r="D3" t="str">
+        <v>8684272100471</v>
+      </c>
+      <c r="E3" t="str">
+        <v>50 ml (1.7 fl.oz)</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Glycine Soja Oil, Rosmarinus Officinalis Leaf Oil, Simmondsia Chinensis Seed Oil, Mentha Piperita Oil, Eucalyptus Globulus Leaf Oil, Menthol, Cocos Nucifera Oil, Equisetum Arvense Extract, Aloe Barbadensis Extract, Lavandula Angustifolia Oil, Triticum Vulgare Germ Oil, Carthamus Tinctorius Seed Oil, Oenothera Biennis Oil, Vitis Vinifera Seed Oil, Benzyl Nicotinate, Prunus Amygdalus Dulcis Oil, Oryza Sativa Bran Oil, Tocopheryl Acetate, Arctium Lappa Root Extract, Glycerin, Apium Graveolens Seed Extract, Ascorbic Acid, Ocimum Basilicum Oil, Pogostemon Cablin Oil, Salvia Officinalis Oil, Silica, Urtica Dioica Extract, Melaleuca Alternifolia Leaf Oil, Ricinus Communis Seed Oil, Malus Domestica Fruit Extract.</v>
+      </c>
+      <c r="G3" t="str">
+        <v>الإدارة تؤكد اكتمال التسجيل، لكن إثبات التسجيل لم يُعثر عليه في الملفات المتاحة</v>
+      </c>
+      <c r="H3" t="str">
+        <v>reconcile INCI (box vs details file) with CEELLO · drop/verify ‘Biotin’ front claim · UAE price (AED) · registration proof copy for this SKU · confirm EAN on current box + GS1 licensee · confirm label company role · brand authorization if requested</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>